<commit_message>
Add MIP Special event problem
</commit_message>
<xml_diff>
--- a/Lectures/Ex2-1-parametric.xlsx
+++ b/Lectures/Ex2-1-parametric.xlsx
@@ -1,32 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Box\_Rosenberg2024\Classes\CEE6410\Fall2024\CEE6410-Rosenberg-GitHub\CEE-6410-Rosenberg\Lectures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B2AC0F7-0B3D-401C-B429-CD42637321EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C1FD1A3-DE2F-4B9D-B2A8-9601C647CBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7270" xr2:uid="{9C63AE14-129A-4C00-AECB-10FA54051378}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{EBE15F71-A306-4597-AF93-14660B5051B2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Table of Contents" sheetId="14" r:id="rId1"/>
-    <sheet name="Scalar" sheetId="13" r:id="rId2"/>
-    <sheet name="A" sheetId="12" r:id="rId3"/>
-    <sheet name="b" sheetId="11" r:id="rId4"/>
-    <sheet name="c" sheetId="10" r:id="rId5"/>
-    <sheet name="DecVars" sheetId="9" r:id="rId6"/>
-    <sheet name="ObjFunc" sheetId="8" r:id="rId7"/>
-    <sheet name="plnt" sheetId="7" r:id="rId8"/>
-    <sheet name="res" sheetId="6" r:id="rId9"/>
-    <sheet name="RES_CONSTRAIN" sheetId="5" r:id="rId10"/>
-    <sheet name="runs" sheetId="4" r:id="rId11"/>
-    <sheet name="ShadowVals" sheetId="3" r:id="rId12"/>
-    <sheet name="TomWatReq" sheetId="2" r:id="rId13"/>
-    <sheet name="X" sheetId="1" r:id="rId14"/>
+    <sheet name="Table of Contents" sheetId="15" r:id="rId1"/>
+    <sheet name="Scalar" sheetId="14" r:id="rId2"/>
+    <sheet name="A" sheetId="13" r:id="rId3"/>
+    <sheet name="b" sheetId="12" r:id="rId4"/>
+    <sheet name="c" sheetId="11" r:id="rId5"/>
+    <sheet name="DecVars" sheetId="10" r:id="rId6"/>
+    <sheet name="ObjFunc" sheetId="9" r:id="rId7"/>
+    <sheet name="plnt" sheetId="8" r:id="rId8"/>
+    <sheet name="res" sheetId="7" r:id="rId9"/>
+    <sheet name="RES_CONSTRAIN" sheetId="6" r:id="rId10"/>
+    <sheet name="runs" sheetId="5" r:id="rId11"/>
+    <sheet name="ShadowVals" sheetId="4" r:id="rId12"/>
+    <sheet name="SLACK" sheetId="3" r:id="rId13"/>
+    <sheet name="TomWatReq" sheetId="2" r:id="rId14"/>
+    <sheet name="X" sheetId="1" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">A!$A$3:$C$9</definedName>
@@ -39,8 +40,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">RES_CONSTRAIN!$A$3:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">runs!$A$3:$A$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">ShadowVals!$A$3:$C$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">TomWatReq!$A$3:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">X!$A$3:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">SLACK!$A$3:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">TomWatReq!$A$3:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">X!$A$3:$E$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,12 +60,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="63">
   <si>
     <t>X</t>
   </si>
@@ -125,18 +130,27 @@
     <t>r4</t>
   </si>
   <si>
+    <t>SLACK</t>
+  </si>
+  <si>
+    <t>Slack value on resource constraints (units of the resource)</t>
+  </si>
+  <si>
+    <t>res</t>
+  </si>
+  <si>
+    <t>Labor</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
     <t>ShadowVals</t>
   </si>
   <si>
     <t>Shadow values of resource constraints ($ per resource)</t>
   </si>
   <si>
-    <t>res</t>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
     <t>Land</t>
   </si>
   <si>
@@ -159,9 +173,6 @@
   </si>
   <si>
     <t>-INF</t>
-  </si>
-  <si>
-    <t>Labor</t>
   </si>
   <si>
     <t>resources</t>
@@ -628,33 +639,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B64B02-138C-484B-ABA6-85150B28B603}">
-  <dimension ref="A1:E15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E934250-D1CA-443E-8C65-D43B9C318B1B}">
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -663,15 +674,15 @@
         <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -680,15 +691,15 @@
         <v>3</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -697,15 +708,15 @@
         <v>2</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -714,15 +725,15 @@
         <v>6</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -731,7 +742,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -739,7 +750,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -748,15 +759,15 @@
         <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -765,7 +776,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -773,7 +784,7 @@
         <v>22</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -782,15 +793,15 @@
         <v>3</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -799,7 +810,7 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -807,7 +818,7 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -816,15 +827,15 @@
         <v>4</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -833,83 +844,101 @@
         <v>6</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>49</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15">
         <v>0</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15">
+      <c r="D15">
         <v>1</v>
       </c>
-      <c r="D15">
+      <c r="E15" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
         <v>2</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" location="A!A1" display="A" xr:uid="{8A49099A-7F21-49A6-85DE-B6E5F8AA0EC7}"/>
-    <hyperlink ref="A3" location="b!A1" display="b" xr:uid="{3335FDE5-2A5B-4EAF-B57D-E3BC09000B5F}"/>
-    <hyperlink ref="A4" location="c!A1" display="c" xr:uid="{220B0919-C455-4702-9CC2-F836192FA99E}"/>
-    <hyperlink ref="A5" location="DecVars!A1" display="DecVars" xr:uid="{650E2446-D96B-4C82-9450-564617D6EAE6}"/>
-    <hyperlink ref="A6" location="ObjFunc!A1" display="ObjFunc" xr:uid="{3F601033-110E-4B8D-AC78-365AD2CA1536}"/>
-    <hyperlink ref="A7" location="plnt!A1" display="plnt" xr:uid="{32243568-5FBF-4365-BCC2-041B7B570ADF}"/>
-    <hyperlink ref="A8" location="Scalar!A1" display="PROFIT" xr:uid="{932230F6-8CB9-4D52-926C-F0310D7D4816}"/>
-    <hyperlink ref="A9" location="res!A1" display="res" xr:uid="{368CB64E-6FC6-4933-85B5-32C401E28C45}"/>
-    <hyperlink ref="A10" location="RES_CONSTRAIN!A1" display="RES_CONSTRAIN" xr:uid="{2B5832E3-6CE7-47AA-AA77-0AF7EA38C3FC}"/>
-    <hyperlink ref="A11" location="runs!A1" display="runs" xr:uid="{CDFA064C-1F10-43A5-B0B1-DA9EE8EA0FBA}"/>
-    <hyperlink ref="A12" location="ShadowVals!A1" display="ShadowVals" xr:uid="{0776BFE6-0185-480F-8C62-D02E701320EF}"/>
-    <hyperlink ref="A13" location="TomWatReq!A1" display="TomWatReq" xr:uid="{31F68952-4569-4894-9B0D-242832B7A694}"/>
-    <hyperlink ref="A14" location="Scalar!A1" display="VPROFIT" xr:uid="{C10F5763-E1B9-42BF-B2AA-736FF085F098}"/>
-    <hyperlink ref="A15" location="X!A1" display="X" xr:uid="{CED8BB13-1C7A-49F3-893A-9E8CF0F6E5AB}"/>
+    <hyperlink ref="A2" location="A!A1" display="A" xr:uid="{89D93CE9-43C0-457E-9AB3-2202EC6D5C2E}"/>
+    <hyperlink ref="A3" location="b!A1" display="b" xr:uid="{DE495CF3-A301-4838-827E-06E7C7E88E4D}"/>
+    <hyperlink ref="A4" location="c!A1" display="c" xr:uid="{67B167D9-56B7-4EF5-89BB-B63353CF1AA1}"/>
+    <hyperlink ref="A5" location="DecVars!A1" display="DecVars" xr:uid="{3D0C0E3A-0B88-4376-90A8-A711FD8D3B9F}"/>
+    <hyperlink ref="A6" location="ObjFunc!A1" display="ObjFunc" xr:uid="{7F6E5990-9785-461B-9669-C0C2E97701C9}"/>
+    <hyperlink ref="A7" location="plnt!A1" display="plnt" xr:uid="{40579D44-395F-4E23-8FA4-9A477A2F3BAD}"/>
+    <hyperlink ref="A8" location="Scalar!A1" display="PROFIT" xr:uid="{2327222D-B4E8-480F-9F1D-FA1BF25494F3}"/>
+    <hyperlink ref="A9" location="res!A1" display="res" xr:uid="{2FBAFEB4-DE0B-43FC-9846-D80DEB736F6D}"/>
+    <hyperlink ref="A10" location="RES_CONSTRAIN!A1" display="RES_CONSTRAIN" xr:uid="{B8DCA2E6-C66D-4A10-9530-CFB00A690B5D}"/>
+    <hyperlink ref="A11" location="runs!A1" display="runs" xr:uid="{13C766FB-0D30-48FC-9C92-A36605CB6C49}"/>
+    <hyperlink ref="A12" location="ShadowVals!A1" display="ShadowVals" xr:uid="{4FC08EEC-9F91-4BAE-9DBC-22E935F33818}"/>
+    <hyperlink ref="A13" location="SLACK!A1" display="SLACK" xr:uid="{6D718536-3B03-4AF0-8444-E2F584B25AD1}"/>
+    <hyperlink ref="A14" location="TomWatReq!A1" display="TomWatReq" xr:uid="{B7A279F6-7179-4188-A23F-2559CCC0C266}"/>
+    <hyperlink ref="A15" location="Scalar!A1" display="VPROFIT" xr:uid="{83ECA12B-1D74-4E69-A643-7FFB43D78102}"/>
+    <hyperlink ref="A16" location="X!A1" display="X" xr:uid="{36C4C102-CC3E-4814-A519-C8A05AF9A54B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9307237-57A7-41EC-AF15-EE2235A5E5F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F862410-5CBA-4B28-8CF8-D7E15D061EBB}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -923,13 +952,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -951,10 +980,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C4">
         <v>2000000</v>
@@ -968,10 +997,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C5">
         <v>12000</v>
@@ -985,10 +1014,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C6">
         <v>10000</v>
@@ -1001,16 +1030,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E6" xr:uid="{D9307237-57A7-41EC-AF15-EE2235A5E5F8}"/>
+  <autoFilter ref="A3:E6" xr:uid="{8F862410-5CBA-4B28-8CF8-D7E15D061EBB}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{C615DCA6-4E00-4F8B-83F0-00001A843690}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{A47883A3-04D1-450D-BACE-E9FE5B526F43}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B6E60F-BA2B-4416-8C30-38F8525578E7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DCB72EA-9481-496A-AF01-17CFE66F8198}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1027,15 +1056,15 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1059,16 +1088,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:A7" xr:uid="{55B6E60F-BA2B-4416-8C30-38F8525578E7}"/>
+  <autoFilter ref="A3:A7" xr:uid="{1DCB72EA-9481-496A-AF01-17CFE66F8198}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{3E2429F4-3579-421A-80E3-F43D5F8E2C4D}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{76E66208-B691-4A21-974D-D9D10D4BB75F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871E5E9A-F0AE-4E5B-8A68-8652A25D63B5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C047B6E-1514-4A70-9DA8-10B0931F7F0C}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1082,13 +1111,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1107,7 +1136,7 @@
         <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4">
         <v>2E-3</v>
@@ -1118,7 +1147,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1129,7 +1158,7 @@
         <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6">
         <v>3.3333333333333322E-3</v>
@@ -1140,7 +1169,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C7">
         <v>0.66666666666666696</v>
@@ -1151,7 +1180,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8">
         <v>7.0000000000000001E-3</v>
@@ -1162,23 +1191,122 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C9">
         <v>2.333333333333333</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C9" xr:uid="{871E5E9A-F0AE-4E5B-8A68-8652A25D63B5}"/>
+  <autoFilter ref="A3:C9" xr:uid="{4C047B6E-1514-4A70-9DA8-10B0931F7F0C}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{8053601D-AAB8-4639-A70E-084C24B43A1C}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{0854B0A5-7519-461C-A5DD-FA4BC514999A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{422B35AF-3A65-49F5-8ECB-790D32730B66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6573AB4F-FD8A-42AD-A825-9BB4070D25BB}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="3" width="15.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5">
+        <v>4166.6666666666679</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8">
+        <v>7500</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:C8" xr:uid="{6573AB4F-FD8A-42AD-A825-9BB4070D25BB}"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{CE47F65B-0F85-42F6-9A7F-2EAA3C1A908D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22148CF7-A633-4C95-9428-0B23680118AC}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1242,16 +1370,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B7" xr:uid="{422B35AF-3A65-49F5-8ECB-790D32730B66}"/>
+  <autoFilter ref="A3:B7" xr:uid="{22148CF7-A633-4C95-9428-0B23680118AC}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{969149F2-4C86-4A36-B2D4-43C47DF4AB55}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{322E44A9-C25E-4983-932B-80CDB513048D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{482822EA-2C6A-4C96-A2F0-5C859C0D0E7B}">
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81085093-6E07-40DB-B662-2B27FB57686F}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1326,16 +1454,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{482822EA-2C6A-4C96-A2F0-5C859C0D0E7B}"/>
+  <autoFilter ref="A3:E5" xr:uid="{81085093-6E07-40DB-B662-2B27FB57686F}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{1A68E684-406B-460E-AC5C-982E4633805A}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{E69CF4E9-E84E-49E5-829B-5110C19CFFF3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE392204-8624-42E3-8CD4-0B03CF80938F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FCC68C2-9C45-4251-80C5-D005C6189740}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1346,18 +1474,18 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -1372,15 +1500,15 @@
         <v>7</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C5">
         <v>27999.999999999996</v>
@@ -1392,12 +1520,12 @@
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
@@ -1412,12 +1540,12 @@
         <v>7</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1432,19 +1560,19 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{B1F19253-9B8A-48E8-ADEF-392A8D099997}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{6E5462BE-079D-44FD-B4FC-657D88480332}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D06AF-7B88-4495-AD8E-CC2A49F8A509}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D1B9530-01BC-4FCC-AD00-C9BE874A91D5}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1458,13 +1586,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1483,7 +1611,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4">
         <v>1000</v>
@@ -1494,7 +1622,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -1505,7 +1633,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -1516,7 +1644,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7">
         <v>500</v>
@@ -1527,7 +1655,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C8">
         <v>3</v>
@@ -1538,23 +1666,23 @@
         <v>10</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="C9">
         <v>2.5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C9" xr:uid="{B41D06AF-7B88-4495-AD8E-CC2A49F8A509}"/>
+  <autoFilter ref="A3:C9" xr:uid="{0D1B9530-01BC-4FCC-AD00-C9BE874A91D5}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{1207E427-6D83-42F4-95EF-D8187E65A663}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{FD8A2379-37FA-4200-A479-B8096ED90CB1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA99D797-EF13-4199-94F5-E5D141427E68}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11EDA8B5-10CC-4FFF-8AF9-032B6AF81B3B}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1568,13 +1696,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1587,7 +1715,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>4000000</v>
@@ -1595,7 +1723,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B5">
         <v>12000</v>
@@ -1603,23 +1731,23 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>17500</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B6" xr:uid="{EA99D797-EF13-4199-94F5-E5D141427E68}"/>
+  <autoFilter ref="A3:B6" xr:uid="{11EDA8B5-10CC-4FFF-8AF9-032B6AF81B3B}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{3AA15614-37FD-40E0-B558-5088B41E42EA}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{618541DF-4DB1-45D5-9B54-790218AB7A67}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5598A2C4-3398-491E-9FC0-9923E8FD954D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E3FE5C-BAAD-4D67-96A4-8A740BD06C85}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1633,13 +1761,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1667,16 +1795,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B5" xr:uid="{5598A2C4-3398-491E-9FC0-9923E8FD954D}"/>
+  <autoFilter ref="A3:B5" xr:uid="{F9E3FE5C-BAAD-4D67-96A4-8A740BD06C85}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{7A7B9E53-9E57-4FA7-890C-5D42A4E71EDB}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{70E8C2F0-F3F7-4267-8609-5B279759CED3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DAA36A-5D15-493A-AF97-506C73FFFF33}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9774D3F9-5397-477E-A886-10CAFD70146B}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1690,13 +1818,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1777,16 +1905,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C9" xr:uid="{20DAA36A-5D15-493A-AF97-506C73FFFF33}"/>
+  <autoFilter ref="A3:C9" xr:uid="{9774D3F9-5397-477E-A886-10CAFD70146B}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{B6813114-24FF-455B-87FA-E3D5FBD14856}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{D43FD346-2D29-4E9C-BC92-801F7AF8E099}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCFB2C6A-CD3F-4DB3-AC01-7A6CA7E0EB1C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C16BC79B-730B-4A17-BE41-AEA99107144F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1800,13 +1928,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1850,16 +1978,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B7" xr:uid="{CCFB2C6A-CD3F-4DB3-AC01-7A6CA7E0EB1C}"/>
+  <autoFilter ref="A3:B7" xr:uid="{C16BC79B-730B-4A17-BE41-AEA99107144F}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{CC256B42-E062-49D4-A7BF-658D4E803279}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{EFF5AC8A-412B-48C3-A54F-07A66775642C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D2817CE-8711-4746-96B2-5DE99BD2C8E7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB16D1EC-0EB5-4CFB-A8BE-126FD755D4A3}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1876,15 +2004,15 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1898,16 +2026,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:A5" xr:uid="{2D2817CE-8711-4746-96B2-5DE99BD2C8E7}"/>
+  <autoFilter ref="A3:A5" xr:uid="{CB16D1EC-0EB5-4CFB-A8BE-126FD755D4A3}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{41393A42-EB28-482E-BFB0-F22BACE50605}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{137607BD-A197-4B81-A5E4-9CB977BE87DB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F540EA30-55BC-4203-90AB-FCB8D6B48B36}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F580FFB-8FC8-4469-9C6D-0566CB1216F7}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1924,36 +2052,36 @@
         <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:A6" xr:uid="{F540EA30-55BC-4203-90AB-FCB8D6B48B36}"/>
+  <autoFilter ref="A3:A6" xr:uid="{2F580FFB-8FC8-4469-9C6D-0566CB1216F7}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{1FD2123F-B600-41A8-831B-7653253F34AF}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{5E20DB5C-7C8A-4EFD-90B2-446C741D1FD8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>